<commit_message>
Add subtitles for two new videos and enhance transcription script
- Added Thai subtitles for two videos: one featuring a discussion about CPU specifications and another sharing an experience related to purchasing a graphics card.
- Enhanced the transcription script to handle larger audio files by processing them in chunks, improving error handling, and allowing for optional export of results in both SRT and JSON formats.
- Updated the script to load environment variables more robustly and added progress indicators for better user experience during transcription.
</commit_message>
<xml_diff>
--- a/references/2026-06-10/viral-cut-2026-06-10.xlsx
+++ b/references/2026-06-10/viral-cut-2026-06-10.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Viral Cuts" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Viral Cuts'!$A$1:$G$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Viral Cuts'!$A$1:$G$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -503,27 +503,27 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>โมเมนต์พี่กับน้องทะเลาะกันกลางไลฟ์!</t>
+          <t>ชิบหายแล้วโรบินฮูช! อาละวาดทั้งทีม</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>01:23:15</t>
+          <t>00:54:53</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>01:27:20</t>
+          <t>00:55:30</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>livestream-2026-06-10.mp4</t>
+          <t>2789194443-194837833-1573b8fc-cffa-4faf-85ee-7ce7abe38671.mp4</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>4 นาที 5 วินาที</t>
+          <t>0 นาที 37 วินาที</t>
         </is>
       </c>
     </row>
@@ -533,37 +533,177 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
+          <t>Chaos</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>CPR ปั๊มปั๊ม! หมอมาแล้วว</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>00:19:08</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>00:19:26</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>2789194443-194837833-1573b8fc-cffa-4faf-85ee-7ce7abe38671.mp4</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>0 นาที 18 วินาที</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="40" customHeight="1">
+      <c r="A4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Plot Twist</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>ผมรู้ทุกอย่าง... เรื่องตัวตนของพี่</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>00:08:36</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>00:08:55</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>2789194443-194837833-1573b8fc-cffa-4faf-85ee-7ce7abe38671.mp4</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>0 นาที 19 วินาที</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="40" customHeight="1">
+      <c r="A5" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
           <t>Interaction</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>แฟนคลับดอนเนท! 10,000 บาทแรกของไลฟ์</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>02:45:10</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>02:48:30</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>livestream-2026-06-10.mp4</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>3 นาที 20 วินาที</t>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>3 ภาษาคุยกันไม่รู้เรื่อง</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>00:42:30</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>00:43:30</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>2789194443-194837833-1573b8fc-cffa-4faf-85ee-7ce7abe38671.mp4</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>1 นาที 0 วินาที</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="40" customHeight="1">
+      <c r="A6" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Humor</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>นกมันกลัว! เสียงปริศนากลางไลฟ์</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>00:34:40</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>00:34:55</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>2789194443-194837833-1573b8fc-cffa-4faf-85ee-7ce7abe38671.mp4</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>0 นาที 15 วินาที</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="40" customHeight="1">
+      <c r="A7" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Emotion</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>โอ้โห เหี้ยฟ้าผ่า! สายฟ้าลั่นสะเทือน</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>01:09:15</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>01:09:30</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>2789194443-194837833-1573b8fc-cffa-4faf-85ee-7ce7abe38671.mp4</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>0 นาที 15 วินาที</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G3"/>
+  <autoFilter ref="A1:G7"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
update reference excel with 1-3 min cuts
</commit_message>
<xml_diff>
--- a/references/2026-06-10/viral-cut-2026-06-10.xlsx
+++ b/references/2026-06-10/viral-cut-2026-06-10.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Viral Cuts" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Viral Cuts'!$A$1:$G$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Viral Cuts'!$A$1:$G$6</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -498,22 +498,22 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Chaos</t>
+          <t>Chaos / Plot Twist</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>ชิบหายแล้วโรบินฮูช! อาละวาดทั้งทีม</t>
+          <t>ลืมซีรี! ลง Windows พัง แล้วเจอหมาบน TikTok</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>00:54:53</t>
+          <t>00:01:40</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>00:55:30</t>
+          <t>00:03:20</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -523,7 +523,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>0 นาที 37 วินาที</t>
+          <t>1 นาที 40 วินาที</t>
         </is>
       </c>
     </row>
@@ -533,22 +533,22 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Chaos</t>
+          <t>Chaos / Humor</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>CPR ปั๊มปั๊ม! หมอมาแล้วว</t>
+          <t>ปวดหัวกับจอย! ตั้งค่าเกมไม่เข้า</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>00:19:08</t>
+          <t>00:03:20</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>00:19:26</t>
+          <t>00:05:10</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
@@ -558,7 +558,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>0 นาที 18 วินาที</t>
+          <t>1 นาที 50 วินาที</t>
         </is>
       </c>
     </row>
@@ -568,22 +568,22 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Plot Twist</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>ผมรู้ทุกอย่าง... เรื่องตัวตนของพี่</t>
+          <t>Chaos / Comedy</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr" s="2">
+        <is>
+          <t>หนีเสือปากจระเข้</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>00:08:36</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>00:08:55</t>
+          <t>00:51:30</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr" s="2">
+        <is>
+          <t>00:53:33</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -593,7 +593,7 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>0 นาที 19 วินาที</t>
+          <t>1 นาที 50 วินาที</t>
         </is>
       </c>
     </row>
@@ -603,22 +603,22 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Interaction</t>
+          <t>Chaos / Educational</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>3 ภาษาคุยกันไม่รู้เรื่อง</t>
+          <t>บอสโหด! ต่อยสามทีตายยกแผง</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>00:42:30</t>
+          <t>01:01:00</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>00:43:30</t>
+          <t>01:04:00</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -628,7 +628,7 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>1 นาที 0 วินาที</t>
+          <t>3 นาที 0 วินาที</t>
         </is>
       </c>
     </row>
@@ -638,22 +638,22 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Humor</t>
+          <t>Plot Twist / Humor</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>นกมันกลัว! เสียงปริศนากลางไลฟ์</t>
+          <t>The Last Airbender มาแล้ว! 4 ผู้เล่นปะทะavatar</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>00:34:40</t>
+          <t>01:17:30</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>00:34:55</t>
+          <t>01:20:00</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -663,47 +663,12 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>0 นาที 15 วินาที</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="40" customHeight="1">
-      <c r="A7" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>Emotion</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>โอ้โห เหี้ยฟ้าผ่า! สายฟ้าลั่นสะเทือน</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>01:09:15</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>01:09:30</t>
-        </is>
-      </c>
-      <c r="F7" s="2" t="inlineStr">
-        <is>
-          <t>2789194443-194837833-1573b8fc-cffa-4faf-85ee-7ce7abe38671.mp4</t>
-        </is>
-      </c>
-      <c r="G7" s="2" t="inlineStr">
-        <is>
-          <t>0 นาที 15 วินาที</t>
+          <t>2 นาที 30 วินาที</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G7"/>
+  <autoFilter ref="A1:G6"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>